<commit_message>
ETradeBenefitHistoryParserTest: assert unvested tranches are skipped
Extends the BenefitHistory.xlsx fixture with two additional Vest Schedule
rows (periods 5 and 6, Vested Qty. = 0, no following Tax Withholding row)
in both G-1001 and G-1002. This mirrors the real Morgan Stanley export
where an active grant has both vested and not-yet-vested tranches and
exercises the parser's per-row vested-qty filter inside an otherwise
vested grant - previously only G-1003 (entirely unvested grant) covered
that path.

Test now also asserts the exact set of vest dates per grant and that
RsuRecord.date == RsuRecord.vestDate, locking in that the parser uses
the corrected Vest Date column from the Vest Schedule row (not any
Event row date).

mvn test: 62 run, 0 failures, 1 skipped.
</commit_message>
<xml_diff>
--- a/src/test/resources/cz/solutions/cockroach/BenefitHistory.xlsx
+++ b/src/test/resources/cz/solutions/cockroach/BenefitHistory.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="75">
   <si>
     <t>Record Type</t>
   </si>
@@ -220,6 +220,12 @@
   </si>
   <si>
     <t>03/20/2026</t>
+  </si>
+  <si>
+    <t>06/20/2026</t>
+  </si>
+  <si>
+    <t>09/20/2026</t>
   </si>
   <si>
     <t>G-1002</t>
@@ -473,7 +479,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP23"/>
+  <dimension ref="A1:AP27"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -753,13 +759,19 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>60</v>
-      </c>
-      <c r="B11" t="s" s="0">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="K11" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="Y11" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="Z11" t="s" s="0">
         <v>69</v>
+      </c>
+      <c r="AG11" t="n" s="0">
+        <v>0.0</v>
       </c>
     </row>
     <row r="12">
@@ -767,33 +779,27 @@
         <v>62</v>
       </c>
       <c r="K12" t="s" s="0">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="Y12" t="n" s="0">
-        <v>1.0</v>
+        <v>6.0</v>
       </c>
       <c r="Z12" t="s" s="0">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="AG12" t="n" s="0">
-        <v>200.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>64</v>
+        <v>60</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>23</v>
       </c>
       <c r="K13" t="s" s="0">
-        <v>69</v>
-      </c>
-      <c r="Y13" t="n" s="0">
-        <v>1.0</v>
-      </c>
-      <c r="AM13" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="AN13" t="n" s="0">
-        <v>3000.0</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14">
@@ -801,13 +807,13 @@
         <v>62</v>
       </c>
       <c r="K14" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Y14" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="Z14" t="s" s="0">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="AG14" t="n" s="0">
         <v>200.0</v>
@@ -818,16 +824,16 @@
         <v>64</v>
       </c>
       <c r="K15" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Y15" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="AM15" t="s" s="0">
         <v>65</v>
       </c>
       <c r="AN15" t="n" s="0">
-        <v>4000.0</v>
+        <v>3000.0</v>
       </c>
     </row>
     <row r="16">
@@ -835,13 +841,13 @@
         <v>62</v>
       </c>
       <c r="K16" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Y16" t="n" s="0">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="Z16" t="s" s="0">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AG16" t="n" s="0">
         <v>200.0</v>
@@ -852,16 +858,16 @@
         <v>64</v>
       </c>
       <c r="K17" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Y17" t="n" s="0">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="AM17" t="s" s="0">
         <v>65</v>
       </c>
       <c r="AN17" t="n" s="0">
-        <v>4400.0</v>
+        <v>4000.0</v>
       </c>
     </row>
     <row r="18">
@@ -869,13 +875,13 @@
         <v>62</v>
       </c>
       <c r="K18" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Y18" t="n" s="0">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="Z18" t="s" s="0">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AG18" t="n" s="0">
         <v>200.0</v>
@@ -886,44 +892,50 @@
         <v>64</v>
       </c>
       <c r="K19" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Y19" t="n" s="0">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="AM19" t="s" s="0">
         <v>65</v>
       </c>
       <c r="AN19" t="n" s="0">
-        <v>5000.0</v>
+        <v>4400.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>60</v>
-      </c>
-      <c r="B20" t="s" s="0">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="K20" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
+      </c>
+      <c r="Y20" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="Z20" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="AG20" t="n" s="0">
+        <v>200.0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="K21" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Y21" t="n" s="0">
-        <v>1.0</v>
-      </c>
-      <c r="Z21" t="s" s="0">
-        <v>71</v>
-      </c>
-      <c r="AG21" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
+      </c>
+      <c r="AM21" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="AN21" t="n" s="0">
+        <v>5000.0</v>
       </c>
     </row>
     <row r="22">
@@ -931,13 +943,13 @@
         <v>62</v>
       </c>
       <c r="K22" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Y22" t="n" s="0">
-        <v>2.0</v>
+        <v>5.0</v>
       </c>
       <c r="Z22" t="s" s="0">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="AG22" t="n" s="0">
         <v>0.0</v>
@@ -945,6 +957,68 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="K23" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="Y23" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="Z23" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="AG23" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="K24" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="K25" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="Y25" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="Z25" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="AG25" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="K26" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="Y26" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="Z26" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="AG26" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
         <v>32</v>
       </c>
     </row>

</xml_diff>